<commit_message>
Clarify verified gain and scenario modes
</commit_message>
<xml_diff>
--- a/public/templates/verified-ai-gain-calculator-sample.xlsx
+++ b/public/templates/verified-ai-gain-calculator-sample.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified AI Gain" sheetId="1" r:id="R48c52f7cc259475e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R77c2143d35054408"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified AI Gain" sheetId="1" r:id="R1c4e945952634c86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R606ca068680740a2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -265,7 +265,7 @@
       </x:c>
       <x:c r="C4" t="n">
         <x:f>Assumptions!B2-Assumptions!B3</x:f>
-        <x:v>3800000000</x:v>
+        <x:v>15000000000</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -277,7 +277,7 @@
       </x:c>
       <x:c r="C5" t="n">
         <x:f>C4*(1-Assumptions!B5)</x:f>
-        <x:v>3230000000</x:v>
+        <x:v>13500000000</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -289,7 +289,7 @@
       </x:c>
       <x:c r="C6" t="n">
         <x:f>MAX(0,C5-Assumptions!B4)</x:f>
-        <x:v>2630000000</x:v>
+        <x:v>12000000000</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -301,7 +301,7 @@
       </x:c>
       <x:c r="C7" t="n">
         <x:f>IF(C6&lt;=0,0,C6*Assumptions!B6)</x:f>
-        <x:v>131500000</x:v>
+        <x:v>600000000</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -313,7 +313,7 @@
       </x:c>
       <x:c r="C8" t="n">
         <x:f>IF(C6&lt;=0,0,C6-C7)</x:f>
-        <x:v>2498500000</x:v>
+        <x:v>11400000000</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -325,7 +325,7 @@
       </x:c>
       <x:c r="C9" t="n">
         <x:f>IF(C6&lt;=0,0,C7/Assumptions!B7)</x:f>
-        <x:v>13150</x:v>
+        <x:v>60000</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -401,7 +401,7 @@
         <x:v>Baseline Annual Process Cost</x:v>
       </x:c>
       <x:c r="B2" t="n">
-        <x:v>12000000000</x:v>
+        <x:v>25000000000</x:v>
       </x:c>
       <x:c r="C2" t="str">
         <x:v>JPY</x:v>
@@ -412,7 +412,7 @@
         <x:v>Post-AI Annual Process Cost</x:v>
       </x:c>
       <x:c r="B3" t="n">
-        <x:v>8200000000</x:v>
+        <x:v>10000000000</x:v>
       </x:c>
       <x:c r="C3" t="str">
         <x:v>JPY</x:v>
@@ -423,7 +423,7 @@
         <x:v>Annual AI Costs</x:v>
       </x:c>
       <x:c r="B4" t="n">
-        <x:v>600000000</x:v>
+        <x:v>1500000000</x:v>
       </x:c>
       <x:c r="C4" t="str">
         <x:v>JPY</x:v>
@@ -434,7 +434,7 @@
         <x:v>Adjustment Rate</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:v>0.15</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="C5" t="str">
         <x:v>%</x:v>
@@ -467,7 +467,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>Only newly created and verified AI productivity gains are eligible.</x:v>
+        <x:v>Default aligns with Medium shortcut: ¥60,000 per employee per year.</x:v>
       </x:c>
       <x:c r="C8" t="str"/>
     </x:row>

</xml_diff>

<commit_message>
Align dashboard with master PPD ledger
</commit_message>
<xml_diff>
--- a/public/templates/verified-ai-gain-calculator-sample.xlsx
+++ b/public/templates/verified-ai-gain-calculator-sample.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified AI Gain" sheetId="1" r:id="R1c4e945952634c86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R606ca068680740a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified AI Gain Ledger" sheetId="1" r:id="R71746042d94440ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" r:id="R32e9f315ca4642f4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -34,13 +34,37 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1">
+  <x:cellXfs count="2">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <xfpb:bag type="Checkbox"/>
+  <xfpb:bag type="XFControls">
+    <xfpb:bagId k="CellControl">0</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplement">
+    <xfpb:bagId k="XFControls">1</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <xfpb:a k="MappedFeaturePropertyBags">
+      <xfpb:bagId>2</xfpb:bagId>
+    </xfpb:a>
+  </xfpb:bag>
+</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -240,7 +264,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
-        <x:v>Verified AI Gain Calculator</x:v>
+        <x:v>Verified AI Gain Ledger</x:v>
       </x:c>
       <x:c r="B1" t="str"/>
       <x:c r="C1" t="str"/>
@@ -258,14 +282,14 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>Gross AI Gain</x:v>
+        <x:v>Eligible Gross Gain</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>Baseline Cost - Post-AI Cost</x:v>
+        <x:v>O + S + Q + M</x:v>
       </x:c>
       <x:c r="C4" t="n">
-        <x:f>Assumptions!B2-Assumptions!B3</x:f>
-        <x:v>15000000000</x:v>
+        <x:f>Inputs!B2+Inputs!B3+Inputs!B4+Inputs!B5</x:f>
+        <x:v>14500000000</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -273,11 +297,11 @@
         <x:v>Adjusted Gross AI Gain</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Gross AI Gain * (1 - Adjustment Rate)</x:v>
+        <x:v>Eligible Gross Gain * (1 - a)</x:v>
       </x:c>
       <x:c r="C5" t="n">
-        <x:f>C4*(1-Assumptions!B5)</x:f>
-        <x:v>13500000000</x:v>
+        <x:f>C4*(1-Inputs!B7)</x:f>
+        <x:v>13050000000</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -285,22 +309,22 @@
         <x:v>Net Verified AI Gain</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Adjusted Gross AI Gain - Annual AI Costs</x:v>
+        <x:v>MAX(0, Adjusted Gross AI Gain - A)</x:v>
       </x:c>
       <x:c r="C6" t="n">
-        <x:f>MAX(0,C5-Assumptions!B4)</x:f>
+        <x:f>MAX(0,C5-Inputs!B6)</x:f>
         <x:v>12000000000</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Pension Allocation</x:v>
+        <x:v>Pension Productivity Dividend Contribution</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Net Verified AI Gain * Allocation Rate</x:v>
+        <x:v>Net Verified AI Gain * d, only when both gates pass</x:v>
       </x:c>
       <x:c r="C7" t="n">
-        <x:f>IF(C6&lt;=0,0,C6*Assumptions!B6)</x:f>
+        <x:f>IF(OR(C6&lt;=0,Inputs!B10=FALSE,Inputs!B11=FALSE),0,C6*Inputs!B8)</x:f>
         <x:v>600000000</x:v>
       </x:c>
     </x:row>
@@ -309,7 +333,7 @@
         <x:v>Company Retained Gain</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>Net Verified AI Gain - Pension Allocation</x:v>
+        <x:v>Net Verified AI Gain - Contribution</x:v>
       </x:c>
       <x:c r="C8" t="n">
         <x:f>IF(C6&lt;=0,0,C6-C7)</x:f>
@@ -318,13 +342,13 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>Pension Value Per Employee</x:v>
+        <x:v>Contribution per Eligible Employee</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>Pension Allocation / Employees Covered</x:v>
+        <x:v>Contribution / E</x:v>
       </x:c>
       <x:c r="C9" t="n">
-        <x:f>IF(C6&lt;=0,0,C7/Assumptions!B7)</x:f>
+        <x:f>IF(C7&lt;=0,0,C7/Inputs!B9)</x:f>
         <x:v>60000</x:v>
       </x:c>
     </x:row>
@@ -333,11 +357,11 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>If Net Verified AI Gain &lt;= 0</x:v>
+        <x:v>No verified gain or failed gate = no pension allocation</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:f>IF(C6&lt;=0,"No verified gain, no pension allocation.","Verified AI gain available for pre-agreed allocation.")</x:f>
-        <x:v>Verified AI gain available for pre-agreed allocation.</x:v>
+        <x:f>IF(C7&lt;=0,"No verified gain, failed gate, or no pre-agreed allocation population: no pension allocation.","Ready for partner confirmation after CFO reconciliation and quality review.")</x:f>
+        <x:v>Ready for partner confirmation after CFO reconciliation and quality review.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -363,7 +387,7 @@
         <x:v>Boundary</x:v>
       </x:c>
       <x:c r="B13" t="str">
-        <x:v>It does not touch existing profit.</x:v>
+        <x:v>PPD does not hold, pool, transfer, invest, or advise on pension assets.</x:v>
       </x:c>
       <x:c r="C13" t="str"/>
     </x:row>
@@ -375,6 +399,15 @@
         <x:v>Only newly created and verified AI productivity gains are eligible.</x:v>
       </x:c>
       <x:c r="C14" t="str"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>Pilot</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>No pension contribution is routed during the measurement pilot.</x:v>
+      </x:c>
+      <x:c r="C15" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -398,10 +431,10 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>Baseline Annual Process Cost</x:v>
+        <x:v>Avoided overtime cost (O)</x:v>
       </x:c>
       <x:c r="B2" t="n">
-        <x:v>25000000000</x:v>
+        <x:v>3000000000</x:v>
       </x:c>
       <x:c r="C2" t="str">
         <x:v>JPY</x:v>
@@ -409,10 +442,10 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Post-AI Annual Process Cost</x:v>
+        <x:v>Avoided outsourcing / contractor cost (S)</x:v>
       </x:c>
       <x:c r="B3" t="n">
-        <x:v>10000000000</x:v>
+        <x:v>2000000000</x:v>
       </x:c>
       <x:c r="C3" t="str">
         <x:v>JPY</x:v>
@@ -420,7 +453,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>Annual AI Costs</x:v>
+        <x:v>Quality / rework / compliance savings (Q)</x:v>
       </x:c>
       <x:c r="B4" t="n">
         <x:v>1500000000</x:v>
@@ -431,45 +464,76 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Adjustment Rate</x:v>
+        <x:v>Evidenced incremental contribution margin (M)</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:v>0.1</x:v>
+        <x:v>8000000000</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>%</x:v>
+        <x:v>JPY</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>Allocation Rate</x:v>
+        <x:v>Incremental AI-related costs (A)</x:v>
       </x:c>
       <x:c r="B6" t="n">
-        <x:v>0.05</x:v>
+        <x:v>1050000000</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>%</x:v>
+        <x:v>JPY</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Employees Covered</x:v>
+        <x:v>Evidence adjustment rate (a)</x:v>
       </x:c>
       <x:c r="B7" t="n">
-        <x:v>10000</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>Employees</x:v>
+        <x:v>%</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>Note</x:v>
-      </x:c>
-      <x:c r="B8" t="str">
-        <x:v>Default aligns with Medium shortcut: ¥60,000 per employee per year.</x:v>
-      </x:c>
-      <x:c r="C8" t="str"/>
+        <x:v>Allocation rate (d)</x:v>
+      </x:c>
+      <x:c r="B8" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>%</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>Eligible employees (E)</x:v>
+      </x:c>
+      <x:c r="B9" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>Employees</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>Quality gate passed</x:v>
+      </x:c>
+      <x:c r="B10" s="1" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C10" t="str"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>Allocation population agreed before measurement</x:v>
+      </x:c>
+      <x:c r="B11" s="1" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C11" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>